<commit_message>
Improve reconciliation logic and move handler_history.json to project root
- Reconcile_Agent_PoC.py: Move Step 2-C (±5% approximate matching) to after
  Step 5 so all exact methods run before any approximate method; add keyword/
  LLM guard for Step 1-B 金額唯一 to prevent semantic mismatches; group Step 5
  batches by (date, bank, memo) to separate same-day same-memo different-bank
  payments
- find_handler.py: Use relative paths; add same-handler shortcut for multiple
  exact-amount history candidates; add EXACT_MIN_FUZZY=0.15 gate to prevent
  low-scoring fuzzy matches; move history file to project root
- Move handler_history.json from 資料1/ to project root
- Update data files (資料/, 資料1/, 資料2/)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/資料/未入帳清單_11505.xlsx
+++ b/資料/未入帳清單_11505.xlsx
@@ -925,11 +925,7 @@
           <t>華邦電現金股息</t>
         </is>
       </c>
-      <c r="J11" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J11" s="14" t="n"/>
       <c r="K11" s="14" t="n"/>
     </row>
     <row r="12" ht="15.6" customHeight="1" s="6">
@@ -21724,7 +21720,11 @@
           <t>英屬開曼群島商</t>
         </is>
       </c>
-      <c r="J474" s="14" t="n"/>
+      <c r="J474" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K474" s="14" t="n"/>
     </row>
     <row r="475" ht="15.6" customHeight="1" s="6">
@@ -21814,11 +21814,7 @@
           <t>00970B</t>
         </is>
       </c>
-      <c r="J476" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J476" s="14" t="n"/>
       <c r="K476" s="14" t="n"/>
     </row>
     <row r="477" ht="15.6" customHeight="1" s="6">
@@ -21953,11 +21949,7 @@
           <t>00904</t>
         </is>
       </c>
-      <c r="J479" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J479" s="14" t="n"/>
       <c r="K479" s="14" t="n"/>
     </row>
     <row r="480" ht="15.6" customHeight="1" s="6">
@@ -22137,11 +22129,7 @@
           <t>兆豐美債收益分配</t>
         </is>
       </c>
-      <c r="J483" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J483" s="14" t="n"/>
       <c r="K483" s="14" t="n"/>
     </row>
     <row r="484" ht="15.6" customHeight="1" s="6">
@@ -22374,7 +22362,11 @@
           <t>寒舍餐旅管理顧問</t>
         </is>
       </c>
-      <c r="J488" s="14" t="n"/>
+      <c r="J488" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K488" s="14" t="n"/>
     </row>
     <row r="489" ht="15.6" customHeight="1" s="6">
@@ -22558,7 +22550,11 @@
           <t>威世波股份有限公</t>
         </is>
       </c>
-      <c r="J492" s="14" t="n"/>
+      <c r="J492" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K492" s="14" t="n"/>
     </row>
     <row r="493" ht="15.6" customHeight="1" s="6">
@@ -22873,7 +22869,11 @@
           <t>禾榮科技股份有限</t>
         </is>
       </c>
-      <c r="J499" s="14" t="n"/>
+      <c r="J499" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K499" s="14" t="n"/>
     </row>
     <row r="500" ht="15.6" customHeight="1" s="6">
@@ -23057,7 +23057,11 @@
           <t>嘉威生活股份有限</t>
         </is>
       </c>
-      <c r="J503" s="14" t="n"/>
+      <c r="J503" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K503" s="14" t="n"/>
     </row>
     <row r="504" ht="15.6" customHeight="1" s="6">
@@ -23102,7 +23106,11 @@
           <t>凱基證券股份有限</t>
         </is>
       </c>
-      <c r="J504" s="14" t="n"/>
+      <c r="J504" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K504" s="14" t="n"/>
     </row>
     <row r="505" ht="15.6" customHeight="1" s="6">
@@ -23511,7 +23519,11 @@
           <t>晶鑽生醫股份有限</t>
         </is>
       </c>
-      <c r="J513" s="14" t="n"/>
+      <c r="J513" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K513" s="14" t="n"/>
     </row>
     <row r="514" ht="15.6" customHeight="1" s="6">
@@ -23744,7 +23756,11 @@
           <t>00715102030701</t>
         </is>
       </c>
-      <c r="J518" s="14" t="n"/>
+      <c r="J518" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K518" s="14" t="n"/>
     </row>
     <row r="519" ht="25.8" customHeight="1" s="6">
@@ -24075,7 +24091,11 @@
           <t>00715102036319</t>
         </is>
       </c>
-      <c r="J525" s="14" t="n"/>
+      <c r="J525" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K525" s="14" t="n"/>
     </row>
     <row r="526" ht="25.8" customHeight="1" s="6">
@@ -25476,7 +25496,11 @@
           <t>雲豹能源科技股份</t>
         </is>
       </c>
-      <c r="J554" s="14" t="n"/>
+      <c r="J554" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K554" s="14" t="n"/>
     </row>
     <row r="555" ht="15.6" customHeight="1" s="6">
@@ -25521,7 +25545,11 @@
           <t>台灣富綢</t>
         </is>
       </c>
-      <c r="J555" s="14" t="n"/>
+      <c r="J555" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K555" s="14" t="n"/>
     </row>
     <row r="556" ht="15.6" customHeight="1" s="6">
@@ -25656,11 +25684,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J558" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J558" s="14" t="n"/>
       <c r="K558" s="14" t="n"/>
     </row>
     <row r="559" ht="15.6" customHeight="1" s="6">
@@ -25705,11 +25729,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J559" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J559" s="14" t="n"/>
       <c r="K559" s="14" t="n"/>
     </row>
     <row r="560" ht="15.6" customHeight="1" s="6">
@@ -25754,11 +25774,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J560" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J560" s="14" t="n"/>
       <c r="K560" s="14" t="n"/>
     </row>
     <row r="561" ht="15.6" customHeight="1" s="6">
@@ -25803,11 +25819,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J561" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J561" s="14" t="n"/>
       <c r="K561" s="14" t="n"/>
     </row>
     <row r="562" ht="15.6" customHeight="1" s="6">
@@ -25852,11 +25864,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J562" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J562" s="14" t="n"/>
       <c r="K562" s="14" t="n"/>
     </row>
     <row r="563" ht="15.6" customHeight="1" s="6">
@@ -25901,11 +25909,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J563" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J563" s="14" t="n"/>
       <c r="K563" s="14" t="n"/>
     </row>
     <row r="564" ht="15.6" customHeight="1" s="6">
@@ -25950,11 +25954,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J564" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J564" s="14" t="n"/>
       <c r="K564" s="14" t="n"/>
     </row>
     <row r="565" ht="15.6" customHeight="1" s="6">
@@ -25999,11 +25999,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J565" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J565" s="14" t="n"/>
       <c r="K565" s="14" t="n"/>
     </row>
     <row r="566" ht="15.6" customHeight="1" s="6">
@@ -26048,11 +26044,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J566" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J566" s="14" t="n"/>
       <c r="K566" s="14" t="n"/>
     </row>
     <row r="567" ht="15.6" customHeight="1" s="6">
@@ -26097,11 +26089,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J567" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J567" s="14" t="n"/>
       <c r="K567" s="14" t="n"/>
     </row>
     <row r="568" ht="15.6" customHeight="1" s="6">
@@ -26146,11 +26134,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J568" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J568" s="14" t="n"/>
       <c r="K568" s="14" t="n"/>
     </row>
     <row r="569" ht="15.6" customHeight="1" s="6">
@@ -26195,11 +26179,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J569" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J569" s="14" t="n"/>
       <c r="K569" s="14" t="n"/>
     </row>
     <row r="570" ht="15.6" customHeight="1" s="6">
@@ -26244,11 +26224,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J570" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J570" s="14" t="n"/>
       <c r="K570" s="14" t="n"/>
     </row>
     <row r="571" ht="15.6" customHeight="1" s="6">
@@ -26293,11 +26269,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J571" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J571" s="14" t="n"/>
       <c r="K571" s="14" t="n"/>
     </row>
     <row r="572" ht="15.6" customHeight="1" s="6">
@@ -26342,11 +26314,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J572" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J572" s="14" t="n"/>
       <c r="K572" s="14" t="n"/>
     </row>
     <row r="573" ht="15.6" customHeight="1" s="6">
@@ -26391,11 +26359,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J573" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J573" s="14" t="n"/>
       <c r="K573" s="14" t="n"/>
     </row>
     <row r="574" ht="15.6" customHeight="1" s="6">
@@ -26440,11 +26404,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J574" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J574" s="14" t="n"/>
       <c r="K574" s="14" t="n"/>
     </row>
     <row r="575" ht="15.6" customHeight="1" s="6">
@@ -26489,11 +26449,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J575" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J575" s="14" t="n"/>
       <c r="K575" s="14" t="n"/>
     </row>
     <row r="576" ht="15.6" customHeight="1" s="6">
@@ -26538,11 +26494,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J576" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J576" s="14" t="n"/>
       <c r="K576" s="14" t="n"/>
     </row>
     <row r="577" ht="15.6" customHeight="1" s="6">
@@ -26587,11 +26539,7 @@
           <t xml:space="preserve">ＨＳＢＣ　ＳＤ　</t>
         </is>
       </c>
-      <c r="J577" s="15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J577" s="14" t="n"/>
       <c r="K577" s="14" t="n"/>
     </row>
     <row r="578" ht="15.6" customHeight="1" s="6">
@@ -28084,7 +28032,11 @@
           <t>台灣國際造船股</t>
         </is>
       </c>
-      <c r="J610" s="14" t="n"/>
+      <c r="J610" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K610" s="14" t="n"/>
     </row>
     <row r="611" ht="15.6" customHeight="1" s="6">
@@ -28268,7 +28220,11 @@
           <t>立普思股份有限公</t>
         </is>
       </c>
-      <c r="J614" s="14" t="n"/>
+      <c r="J614" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="K614" s="14" t="n"/>
     </row>
     <row r="615" ht="15.6" customHeight="1" s="6">

</xml_diff>